<commit_message>
feat: Add Mobile E2E Pixel 7 automation, security vulnerability test suite, and hide Appium workflow
</commit_message>
<xml_diff>
--- a/automation/web/reports/Automation_Test_Report.xlsx
+++ b/automation/web/reports/Automation_Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
   <si>
     <t>Metric</t>
   </si>
@@ -66,6 +66,24 @@
   </si>
   <si>
     <t>TC_UI_004: Should verify UI theme tokens and responsive navigation elements</t>
+  </si>
+  <si>
+    <t>Carcinova Mobile Native E2E Test Suite (Pixel 7 Emulation)</t>
+  </si>
+  <si>
+    <t>TC_MOB_001: Should login and display mobile top app bar with hamburger icon</t>
+  </si>
+  <si>
+    <t>TC_MOB_002: Should toggle open mobile navigation drawer and display Carcinova branding</t>
+  </si>
+  <si>
+    <t>TC_MOB_003: Should verify mobile touch targets meet 48dp minimum standard</t>
+  </si>
+  <si>
+    <t>TC_MOB_004: Should navigate to Case History on mobile and show card list view</t>
+  </si>
+  <si>
+    <t>TC_MOB_005: Should navigate to Settings on mobile and verify stacked account layout</t>
   </si>
 </sst>
 </file>
@@ -462,7 +480,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -470,7 +488,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -494,7 +512,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>6032</v>
+        <v>19798</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -513,7 +531,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -546,7 +564,7 @@
         <v>13</v>
       </c>
       <c r="D2">
-        <v>4147</v>
+        <v>4288</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -560,7 +578,7 @@
         <v>13</v>
       </c>
       <c r="D3">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -574,7 +592,7 @@
         <v>13</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -588,7 +606,7 @@
         <v>13</v>
       </c>
       <c r="D5">
-        <v>1180</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -602,7 +620,77 @@
         <v>13</v>
       </c>
       <c r="D6">
-        <v>12</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <v>7272</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10">
+        <v>2215</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11">
+        <v>2210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>